<commit_message>
chore: replace README sheet with blank fillable template
Catering.xlsx and Activities.xlsx now open on a blank Template page
(3 vendor blocks, Item/Cost price/Amount/Sum, Subtotal/Delivery Fee/
Platform Fee/Pretax Subtotal/Tax/Tip/TOTAL formulas) instead of a
description page, so future organizers can copy it for a new event.
</commit_message>
<xml_diff>
--- a/past-proposals/quotes/Activities.xlsx
+++ b/past-proposals/quotes/Activities.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bouldering &amp; Social Mixer (Feb " sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,13 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
@@ -76,12 +83,17 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5233"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -114,65 +126,64 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -540,24 +551,397 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Activities — Vendor Quote History</t>
+          <t>TEMPLATE — copy this sheet for a new event</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Each page below is one event, reproduced from the original quote spreadsheets (lists-of-quotes/) with vendors side by side and the same subtotal / delivery / tax / tip formulas as the source.</t>
-        </is>
+          <t>Vendor 1 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Vendor 2 Name</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Vendor 3 Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Cost price</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Cost price</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Cost price</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="D5">
+        <f>B5*C5</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>F5*G5</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>J5*K5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>F6*G6</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>J6*K6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7">
+        <f>B7*C7</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>F7*G7</f>
+        <v/>
+      </c>
+      <c r="L7">
+        <f>J7*K7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8">
+        <f>B8*C8</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>F8*G8</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>J8*K8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9">
+        <f>B9*C9</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>F9*G9</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>J9*K9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10">
+        <f>B10*C10</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>F10*G10</f>
+        <v/>
+      </c>
+      <c r="L10">
+        <f>J10*K10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11">
+        <f>B11*C11</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>F11*G11</f>
+        <v/>
+      </c>
+      <c r="L11">
+        <f>J11*K11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12">
+        <f>B12*C12</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>F12*G12</f>
+        <v/>
+      </c>
+      <c r="L12">
+        <f>J12*K12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13">
+        <f>B13*C13</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>F13*G13</f>
+        <v/>
+      </c>
+      <c r="L13">
+        <f>J13*K13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14">
+        <f>B14*C14</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>F14*G14</f>
+        <v/>
+      </c>
+      <c r="L14">
+        <f>J14*K14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Subtotal Food</t>
+        </is>
+      </c>
+      <c r="D16">
+        <f>SUM(D5:D14)</f>
+        <v/>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Subtotal Food</t>
+        </is>
+      </c>
+      <c r="H16">
+        <f>SUM(H5:H14)</f>
+        <v/>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Subtotal Food</t>
+        </is>
+      </c>
+      <c r="L16">
+        <f>SUM(L5:L14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Delivery Fee</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Delivery Fee</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Delivery Fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Platform Fee</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Platform Fee</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Platform Fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Pretax Subtotal</t>
+        </is>
+      </c>
+      <c r="D20">
+        <f>SUM(D16:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Pretax Subtotal</t>
+        </is>
+      </c>
+      <c r="H20">
+        <f>SUM(H16:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Pretax Subtotal</t>
+        </is>
+      </c>
+      <c r="L20">
+        <f>SUM(L16:L19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Taxes (13%)</t>
+        </is>
+      </c>
+      <c r="D21">
+        <f>D20*0.13</f>
+        <v/>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Taxes (13%)</t>
+        </is>
+      </c>
+      <c r="H21">
+        <f>H20*0.13</f>
+        <v/>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Taxes (13%)</t>
+        </is>
+      </c>
+      <c r="L21">
+        <f>L20*0.13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D22">
+        <f>SUM(D20:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="H22">
+        <f>SUM(H20:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L22">
+        <f>SUM(L20:L21)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -596,295 +980,295 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>— Bouldering Gym —</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Basecamp Climbing @ Queen Street</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Axe Throwing @ BATL Grounds</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Bowling @ The Ballroom Bowl Yorkville</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Cost price</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Sum</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Cost price</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Sum</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Cost price</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>Sum</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Day Pass (Student)</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="12">
         <f>C7*B7</f>
         <v/>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Play 2 Bundle (90min)</t>
         </is>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <v>37.99</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="14">
         <f>G7*F7</f>
         <v/>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>Adult Peak (1h)</t>
         </is>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="14" t="n">
         <v>32.5</v>
       </c>
-      <c r="K7" s="14" t="n">
+      <c r="K7" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="L7" s="13">
+      <c r="L7" s="14">
         <f>K7*J7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Shoe Rental</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="12">
         <f>C8*B8</f>
         <v/>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I8" s="16" t="inlineStr">
         <is>
           <t>Adult Peak (2h)</t>
         </is>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="14">
         <f>J7*2</f>
         <v/>
       </c>
-      <c r="K8" s="14" t="n">
+      <c r="K8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="13">
+      <c r="L8" s="14">
         <f>K8*J8</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Subtotal Food</t>
         </is>
       </c>
-      <c r="D17" s="17">
+      <c r="D17" s="18">
         <f>SUM(D7:D15)</f>
         <v/>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="19">
         <f> Sum(H7:H16)</f>
         <v/>
       </c>
-      <c r="I17" s="12" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="L17" s="18">
+      <c r="L17" s="19">
         <f> Sum(L7:L15)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Delivery Fee</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Pretax Subtotal</t>
         </is>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="18">
         <f>SUM(D17:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>Pretax Subtotal</t>
         </is>
       </c>
-      <c r="H20" s="18">
+      <c r="H20" s="19">
         <f>SUM(H17:H19)</f>
         <v/>
       </c>
-      <c r="I20" s="12" t="inlineStr">
+      <c r="I20" s="13" t="inlineStr">
         <is>
           <t>Pretax Subtotal</t>
         </is>
       </c>
-      <c r="L20" s="18">
+      <c r="L20" s="19">
         <f>SUM(L17:L19)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Taxes (13%)</t>
         </is>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="12">
         <f>D20*0.13</f>
         <v/>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>Taxes (13%)</t>
         </is>
       </c>
-      <c r="H21" s="13">
+      <c r="H21" s="14">
         <f>H20*0.13</f>
         <v/>
       </c>
-      <c r="I21" s="15" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Taxes (13%)</t>
         </is>
       </c>
-      <c r="L21" s="13">
+      <c r="L21" s="14">
         <f>L20*0.13</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL </t>
         </is>
       </c>
-      <c r="D23" s="22">
+      <c r="D23" s="23">
         <f>SUM(D20:D22)</f>
         <v/>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL </t>
         </is>
       </c>
-      <c r="H23" s="23">
+      <c r="H23" s="24">
         <f>SUM(H20:H22)</f>
         <v/>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>TOTAL (FOOD)</t>
         </is>
       </c>
-      <c r="L23" s="23">
+      <c r="L23" s="24">
         <f>SUM(L20:L22)</f>
         <v/>
       </c>

</xml_diff>